<commit_message>
docs(rapids): renumber drifted signal-contract citations (rapids TASK-022)
Workstream A residue: bf5db01b7 line drift broke 23 citation tuples in
gen_rapids_signal_contracts_kmaps.py (exit 1). Renumbered mechanically;
8 tuples needed snippet updates where the RTL text itself changed
(w_eff_drain_size, r_res_ch/r_res_size, r_d_active, w_drain_data_available_acct,
w_channel_has_space/w_space_now, s_axis_tready, w_transfer_complete), prose
STR_RENG refs 580->656 and STR_WENG 387->401. Generator exits 0; workbook
regenerated. TASK-022 records Workstream A done-by-bf5db01b7 (split
correction 40/24), the Done-when dir list, and the axi_read_engine
adjacent gap.
</commit_message>
<xml_diff>
--- a/projects/components/dma-ip/rapids/docs/rapids_signal_contracts.xlsx
+++ b/projects/components/dma-ip/rapids/docs/rapids_signal_contracts.xlsx
@@ -606,12 +606,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>A drain_req must only assert when the drain controller's own data_available &gt;= drain_size. The module asserts this itself (projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176) but only as a simulation $error.</t>
+          <t>A drain_req must only assert when the drain controller's own data_available &gt;= drain_size. The module asserts this itself (projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176) but only as a simulation $error.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:222, wired at projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:157. DEFECT: the qualifying comparison uses an INFLATED view -- see projects/components/dmas/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:222, wired at projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:157. DEFECT: the qualifying comparison uses an INFLATED view -- see projects/components/dma-ip/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md.</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:223, consumed projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:223, consumed projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229 -- THE DEFECT. Over-count is 0..4 (projects/components/dmas/rapids/rtl/fub_beats/latency_bridge_beats.sv:185). STREAM carried the identical line and removed it; see projects/components/dmas/stream/rtl/fub/sram_controller_unit.sv:282-307 for the prohibition and the deadlock it caused. projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:229 is the same line, unfixed.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229 -- THE DEFECT. Over-count is 0..4 (projects/components/dma-ip/rapids/rtl/fub_beats/latency_bridge_beats.sv:185). STREAM carried the identical line and removed it; see projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:282-307 for the prohibition and the deadlock it caused. projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:229 is the same line, unfixed.</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:229, projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:251.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:229, projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:251.</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142 driven, discarded at projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:159. STREAM also leaves it unconnected -- stream fixes the problem upstream instead, at projects/components/dmas/stream/rtl/fub/sram_controller_unit.sv:307 and projects/components/dmas/stream/rtl/fub/axi_write_engine.sv:387.</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142 driven, discarded at projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:159. STREAM also leaves it unconnected -- stream fixes the problem upstream instead, at projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:307 and projects/components/dma-ip/stream/rtl/fub/axi_write_engine.sv:387.</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>src_data_path_axis_beats / drain_ctrl_beats - drain grant (projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv)</t>
+          <t>src_data_path_axis_beats / drain_ctrl_beats - drain grant (projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv)</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TARGET: rapids TASK-002 item 3, the DRAIN_SIZE&gt;1 source beat drop (projects/components/dmas/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md). The first map is the important one -- it is a map whose 1-cells include cells that should be impossible, and the axis that would have excluded them is not an input to the decision at all.</t>
+          <t>TARGET: rapids TASK-002 item 3, the DRAIN_SIZE&gt;1 source beat drop (projects/components/dma-ip/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md). The first map is the important one -- it is a map whose 1-cells include cells that should be impossible, and the axis that would have excluded them is not an input to the decision at all.</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:197</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:197</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: HEALTHY: every green cell would sit at fifo_ge_size=1 -- a reservation only ever committed against beats that are really in the drain controller. ACTUAL: fifo_ge_size does not appear in the expression at all, so the map is INDEPENDENT of it: of the two green cells, one sits at fifo_ge_size=1 (correct) and one at fifo_ge_size=0 -- (avail_ge_size=1, fifo_ge_size=0, should_advance=1, req_pending=1) -- and THAT cell is the defect. In it the arbiter commits a cfg_drain_size reservation while the drain controller holds less than that, drain_ctrl_beats advances rd_ptr by the full size anyway (projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102, gated only on !r_rd_empty), and rd_ptr overshoots wr_ptr. Per the module's own comment (projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:156) that corruption is PERMANENT. Those cells are reachable exactly when bridge_occupancy &gt; 0, which is the steady state whenever the bridge holds its prefetch. At cfg_drain_size == 1 the !r_rd_empty gate absorbs the whole discrepancy, which is why DRAIN_SIZE=1 is clean and is the shipped workaround.</t>
+          <t>CHECK BY INSPECTION: HEALTHY: every green cell would sit at fifo_ge_size=1 -- a reservation only ever committed against beats that are really in the drain controller. ACTUAL: fifo_ge_size does not appear in the expression at all, so the map is INDEPENDENT of it: of the two green cells, one sits at fifo_ge_size=1 (correct) and one at fifo_ge_size=0 -- (avail_ge_size=1, fifo_ge_size=0, should_advance=1, req_pending=1) -- and THAT cell is the defect. In it the arbiter commits a cfg_drain_size reservation while the drain controller holds less than that, drain_ctrl_beats advances rd_ptr by the full size anyway (projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102, gated only on !r_rd_empty), and rd_ptr overshoots wr_ptr. Per the module's own comment (projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:156) that corruption is PERMANENT. Those cells are reachable exactly when bridge_occupancy &gt; 0, which is the steady state whenever the bridge holds its prefetch. At cfg_drain_size == 1 the !r_rd_empty gate absorbs the whole discrepancy, which is why DRAIN_SIZE=1 is clean and is the shipped workaround.</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:197 (view built at projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229)</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:197 (view built at projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229)</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:162, consumed projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:162, consumed projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:102</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:169</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:169</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229, projects/components/dmas/rapids/rtl/fub_beats/latency_bridge_beats.sv:185</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229, projects/components/dma-ip/rapids/rtl/fub_beats/latency_bridge_beats.sv:185</t>
         </is>
       </c>
     </row>
@@ -980,14 +980,14 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:169</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:169</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DEPENDS ONLY ON: these four. cfg_drain_size is a configuration constant held across the transfer; r_arb_grant_id/check_ch select WHICH channel is examined, not whether a grant fires; r_drain_remaining gates the decrement path, not this one. Critically, NOTHING in the cone reads the drain controller's own not-empty flag -- it is driven (projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142) and then discarded unconnected (projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:159).</t>
+          <t>DEPENDS ONLY ON: these four. cfg_drain_size is a configuration constant held across the transfer; r_arb_grant_id/check_ch select WHICH channel is examined, not whether a grant fires; r_drain_remaining gates the decrement path, not this one. Critically, NOTHING in the cone reads the drain controller's own not-empty flag -- it is driven (projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142) and then discarded unconnected (projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:159).</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:101</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:101</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: The map is INDEPENDENT of size_gt_avail: the pointer advances in both size_gt_avail cells of the v=1,ne=1 column. The $error at projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176 fires in exactly one of those two cells and changes nothing -- it is a DETECTOR, not a guard, and it is wrapped in translate_off so it exists only in simulation. No DRAIN_SIZE&gt;1 configuration is present in the checked-in RAPIDS collateral and no over-drain report exists anywhere in the tree, but the known issue records a DRAIN_SIZE=8 A/B run in sim (projects/components/dmas/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md), so whether this $error has ever actually fired is UNESTABLISHED. Re-running that A/B and grepping for it is the cheapest available confirmation of the whole mechanism. HEALTHY would be a map that is 0 wherever size_gt_avail=1.</t>
+          <t>CHECK BY INSPECTION: The map is INDEPENDENT of size_gt_avail: the pointer advances in both size_gt_avail cells of the v=1,ne=1 column. The $error at projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176 fires in exactly one of those two cells and changes nothing -- it is a DETECTOR, not a guard, and it is wrapped in translate_off so it exists only in simulation. No DRAIN_SIZE&gt;1 configuration is present in the checked-in RAPIDS collateral and no over-drain report exists anywhere in the tree, but the known issue records a DRAIN_SIZE=8 A/B run in sim (projects/components/dma-ip/rapids/known_issues/active/drain_size_gt1_source_beat_drop.md), so whether this $error has ever actually fired is UNESTABLISHED. Re-running that A/B and grepping for it is the cheapest available confirmation of the whole mechanism. HEALTHY would be a map that is 0 wherever size_gt_avail=1.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:78 (wired projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:157)</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:78 (wired projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:157)</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:142</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: The cells at arb_active=1, avail_zero=1, rem_zero=0 are ABANDONMENT: the arbiter drops a grant while r_drain_remaining is still non-zero. The reservation for that grant already advanced the read pointer by the full cfg_drain_size, so the beats between what was reserved and what was actually moved are skipped -- they are never emitted and never recovered. This is the second half of the loss mechanism and it is why the shortfall is not a clean multiple of DRAIN_SIZE. Note also that the decrement of r_drain_remaining sits in the ELSE of this condition (projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:204), so on any advancing cycle a beat can leave without being counted against the block.</t>
+          <t>CHECK BY INSPECTION: The cells at arb_active=1, avail_zero=1, rem_zero=0 are ABANDONMENT: the arbiter drops a grant while r_drain_remaining is still non-zero. The reservation for that grant already advanced the read pointer by the full cfg_drain_size, so the beats between what was reserved and what was actually moved are skipped -- they are never emitted and never recovered. This is the second half of the loss mechanism and it is why the shortfall is not a clean multiple of DRAIN_SIZE. Note also that the decrement of r_drain_remaining sits in the ELSE of this condition (projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:204), so on any advancing cycle a beat can leave without being counted against the block.</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:180</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:181</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:181</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:229</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:229</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:182</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:182</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:251, projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/src_data_path_axis_beats.sv:251, projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/stream/rtl/fub/sram_controller_unit.sv:282-307</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:282-307</t>
         </is>
       </c>
     </row>
@@ -1647,12 +1647,12 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>data_available ONLY (projects/components/dmas/stream/rtl/fub/sram_controller_unit.sv:307)</t>
+          <t>data_available ONLY (projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:307)</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>data_available + bridge_occupancy (projects/components/dmas/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229)</t>
+          <t>data_available + bridge_occupancy (projects/components/dma-ip/rapids/rtl/macro_beats/src_sram_controller_unit_beats.sv:229)</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>yes, as a prohibition with the deadlock it caused (projects/components/dmas/stream/rtl/fub/sram_controller_unit.sv:282-301)</t>
+          <t>yes, as a prohibition with the deadlock it caused (projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:282-301)</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>w_effective_avail = avail - in-flight drains (projects/components/dmas/stream/rtl/fub/axi_write_engine.sv:387)</t>
+          <t>w_effective_avail = avail - in-flight drains (projects/components/dma-ip/stream/rtl/fub/axi_write_engine.sv:401)</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>identical module, identical over-drain $error (projects/components/dmas/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176)</t>
+          <t>identical module, identical over-drain $error (projects/components/dma-ip/rapids/rtl/fub_beats/drain_ctrl_beats.sv:176)</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>same unfixed line at projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:229</t>
+          <t>same unfixed line at projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:229</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1837,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>A beat accepted on AXIS must be stored. The only real store is fill_valid &amp;&amp; fill_ready (projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:184-185, the FIFO's own wr_ready), so any accepted beat for which fill_ready was low is consumed off the network and lost.</t>
+          <t>A beat accepted on AXIS must be stored. The only real store is fill_valid &amp;&amp; fill_ready (projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:225-226, the FIFO's own wr_ready), so any accepted beat for which fill_ready was low is consumed off the network and lost.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204-205 -- THE DEFECT CANDIDATE. See the K-map sheet for which cell and what is not yet established about reaching it.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204-205 -- THE DEFECT CANDIDATE. See the K-map sheet for which cell and what is not yet established about reaching it.</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189; discarded ready at projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:126; allocator gating at projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:76 and projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:86.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189; discarded ready at projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:136; allocator gating at projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:76 and projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:86.</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219-229. STREAM has no equivalent counter at all (zero occurrences in stream/rtl); it registers its alloc request and proves the contract instead -- projects/components/dmas/stream/rtl/fub/axi_read_engine.sv:580, inside an `ifdef FORMAL` block.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219-229. STREAM has no equivalent counter at all (zero occurrences in stream/rtl); it registers its alloc request and proves the contract instead -- projects/components/dma-ip/stream/rtl/fub/axi_read_engine.sv:656, inside an `ifdef FORMAL` block.</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:236. ALLOC_SIZE is an 8-bit rw CSR field defaulting to 0x10, so 1 is a writable value.</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:314. ALLOC_SIZE is an 8-bit rw CSR field defaulting to 0x10, so 1 is a writable value.</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:234.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:234.</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>snk_data_path_axis_beats - AXIS ingress admission (projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv)</t>
+          <t>snk_data_path_axis_beats - AXIS ingress admission (projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv)</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: HEALTHY: every green cell would sit at fill_ready=1, because the only actual store is fill_valid &amp;&amp; fill_ready (projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:184-185). ACTUAL: the single green cell at fill_ready=0 (alloc_req=1, pending_gt0=0) accepts an AXIS beat while the FIFO is backpressuring. The handshake completes, the beat is consumed off the network, and nothing stores it -- and projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:234 then counts it as received. NOT YET ESTABLISHED: whether that cell is reachable in practice. It needs fill_ready=0 simultaneously with fill_space_free &gt;= cfg_alloc_size, and those are two DIFFERENT counters -- the FIFO's own occupancy versus alloc_ctrl's allocation accounting (projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:141), which is released only when data leaves the latency bridge. Proving or excluding that co-occurrence is the open question this map poses; a directed test driving AXIS into a backpressured channel would settle it.</t>
+          <t>CHECK BY INSPECTION: HEALTHY: every green cell would sit at fill_ready=1, because the only actual store is fill_valid &amp;&amp; fill_ready (projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:225-226). ACTUAL: the single green cell at fill_ready=0 (alloc_req=1, pending_gt0=0) accepts an AXIS beat while the FIFO is backpressuring. The handshake completes, the beat is consumed off the network, and nothing stores it -- and projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:234 then counts it as received. NOT YET ESTABLISHED: whether that cell is reachable in practice. It needs fill_ready=0 simultaneously with fill_space_free &gt;= cfg_alloc_size, and those are two DIFFERENT counters -- the FIFO's own occupancy versus alloc_ctrl's allocation accounting (projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:141), which is released only when data leaves the latency bridge. Proving or excluding that co-occurrence is the open question this map poses; a directed test driving AXIS into a backpressured channel would settle it.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:185</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:226</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:185, projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:185, projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:189</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:197</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:197</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:197</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:197</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:198</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:198</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:199</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:199</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:185</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:185</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2548,7 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: The map is INDEPENDENT of alloc_granted, which is the finding. alloc_ctrl advances its pointer only on w_write &amp;&amp; !r_wr_full (projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:76, projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:86), so a request arriving while the allocator is full is silently dropped -- yet r_pending_alloc is credited the full fill_alloc_size regardless. The two green cells at alloc_granted=0 are where the datapath believes it holds space the allocator never gave it. HEALTHY would be a map that is 0 wherever alloc_granted=0, which requires routing wr_ready back -- it is driven and available, just not connected.</t>
+          <t>CHECK BY INSPECTION: The map is INDEPENDENT of alloc_granted, which is the finding. alloc_ctrl advances its pointer only on w_write &amp;&amp; !r_wr_full (projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:76, projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:86), so a request arriving while the allocator is full is silently dropped -- yet r_pending_alloc is credited the full fill_alloc_size regardless. The two green cells at alloc_granted=0 are where the datapath believes it holds space the allocator never gave it. HEALTHY would be a map that is 0 wherever alloc_granted=0, which requires routing wr_ready back -- it is driven and available, just not connected.</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:219</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:222</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:222</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:137, discarded at projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:126</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/alloc_ctrl_beats.sv:137, discarded at projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:136</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_unit_beats.sv:126</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/sram_controller_unit.sv:136</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/stream/rtl/fub/axi_read_engine.sv:580</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/axi_read_engine.sv:656</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>r_pending_alloc, credited on request (projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:225)</t>
+          <t>r_pending_alloc, credited on request (projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:225)</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>yes, and PROVEN: alloc_req |-&gt; $past(arvalid &amp;&amp; arready) (projects/components/dmas/stream/rtl/fub/axi_read_engine.sv:580, inside `ifdef FORMAL`)</t>
+          <t>yes, and PROVEN: alloc_req |-&gt; $past(arvalid &amp;&amp; arready) (projects/components/dma-ip/stream/rtl/fub/axi_read_engine.sv:656, inside `ifdef FORMAL`)</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>NO: s_axis_tready ORs in fill_alloc_req (projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204)</t>
+          <t>NO: s_axis_tready ORs in fill_alloc_req (projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_axis_beats.sv:204)</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>scheduler_beats - completion gating and timeout escalation (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv)</t>
+          <t>scheduler_beats - completion gating and timeout escalation (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv)</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TARGET: rapids TASK-002 item 4. Unlike the alloc/drain FUBs (byte-identical to STREAM's), this module DIVERGED: 1150 lines against STREAM's 1390. Map 1 is where the divergence lives, and it is the cone of the resolved wedge in projects/components/dmas/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md.</t>
+          <t>TARGET: rapids TASK-002 item 4. Unlike the alloc/drain FUBs (byte-identical to STREAM's), this module DIVERGED: 1150 lines against STREAM's 1390. Map 1 is where the divergence lives, and it is the cone of the resolved wedge in projects/components/dma-ip/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md.</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:418</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:418</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: The map is INDEPENDENT of write_issued, which is the divergence. STREAM exits this state on ISSUE (projects/components/dmas/stream/rtl/fub/scheduler.sv:909, w_transfer_complete = w_read_complete &amp;&amp; w_write_issued) and defers the commit-wait to CH_COMPLETE, and only for the LAST descriptor (projects/components/dmas/stream/rtl/fub/scheduler.sv:542). RAPIDS waits for COMMITS here, on EVERY descriptor (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:776), and its CH_COMPLETE carries no commit gate at all. Two consequences. (1) Chain throughput: RAPIDS cannot advance to the next descriptor until the current one's B responses land; STREAM streams through. (2) A lost commit surfaces on ANY descriptor in RAPIDS rather than only the last. NOT a tolerance difference: under a lost commit NEITHER design recovers -- write_committed never reaches 1, no green cell is ever entered, the channel never reaches CH_IDLE and scheduler_idle (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:1105) never asserts. That is the wedge recorded in projects/components/dmas/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md (ILA: r_write_beats_to_commit=1, r_write_beats_remaining=0).</t>
+          <t>CHECK BY INSPECTION: The map is INDEPENDENT of write_issued, which is the divergence. STREAM exits this state on ISSUE (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:909, w_transfer_complete = w_read_complete &amp;&amp; w_write_issued) and defers the commit-wait to CH_COMPLETE, and only for the LAST descriptor (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:542). RAPIDS waits for COMMITS here, on EVERY descriptor (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:776), and its CH_COMPLETE carries no commit gate at all. Two consequences. (1) Chain throughput: RAPIDS cannot advance to the next descriptor until the current one's B responses land; STREAM streams through. (2) A lost commit surfaces on ANY descriptor in RAPIDS rather than only the last. NOT a tolerance difference: under a lost commit NEITHER design recovers -- write_committed never reaches 1, no green cell is ever entered, the channel never reaches CH_IDLE and scheduler_idle (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:1105) never asserts. That is the wedge recorded in projects/components/dma-ip/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md (ILA: r_write_beats_to_commit=1, r_write_beats_remaining=0).</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:771</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:771</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/stream/rtl/fub/scheduler.sv:902</t>
+          <t>projects/components/dma-ip/stream/rtl/fub/scheduler.sv:902</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:775</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:775</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:779</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:779</t>
         </is>
       </c>
     </row>
@@ -3027,14 +3027,14 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:775, projects/components/dmas/stream/rtl/fub/scheduler.sv:902</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:775, projects/components/dma-ip/stream/rtl/fub/scheduler.sv:902</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>DEPENDS ONLY ON: these four for a DATA descriptor. The timeout path reaches the FSM through a separate w_hard_error/w_timeout_escalate branch evaluated BEFORE this case (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:978); channel reset overrides both.</t>
+          <t>DEPENDS ONLY ON: these four for a DATA descriptor. The timeout path reaches the FSM through a separate w_hard_error/w_timeout_escalate branch evaluated BEFORE this case (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:978); channel reset overrides both.</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:858</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:858</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: The issue-count gate is what stops a spurious garbage AW during the commit-wait (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:853-857). Note the !w_write_complete term is LOGICALLY REDUNDANT here: beats_to_issue=1 already forces write_committed=0 (see the relation), so it can never be the deciding term -- every cell where it would matter is marked X. It is belt-and-braces, not live logic, and a future reader should not assume removing it changes behaviour. STREAM carries the same 5-term conjunction with a near-identical comment (projects/components/dmas/stream/rtl/fub/scheduler.sv:1004-1008), so this gate did NOT diverge.</t>
+          <t>CHECK BY INSPECTION: The issue-count gate is what stops a spurious garbage AW during the commit-wait (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:853-857). Note the !w_write_complete term is LOGICALLY REDUNDANT here: beats_to_issue=1 already forces write_committed=0 (see the relation), so it can never be the deciding term -- every cell where it would matter is marked X. It is belt-and-braces, not live logic, and a future reader should not assume removing it changes behaviour. STREAM carries the same 5-term conjunction with a near-identical comment (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:1004-1008), so this gate did NOT diverge.</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:858</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:858</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:859</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:859</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:860</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:860</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:861</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:861</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:862</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:862</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:775, projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:859</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:775, projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:859</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: Escalation drives the channel into sticky CH_ERROR (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:380), so the green cells are fatal transitions. The map is INDEPENDENT of timeout_enable, and that is worth a look: strikes are cleared only by channel reset, by reaching CH_IDLE, or by real write progress (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:932-936) -- never by the enable bit going low. So a channel that has already accumulated strikes and then has cfg_sched_timeout_enable cleared by software still has w_timeout_escalate asserted and still wedges into CH_ERROR. NOT YET ESTABLISHED whether any host sequence actually clears enable mid-transfer; the map states the exposure rather than asserting the bug. A directed test that raises strikes, clears enable, and checks the channel does not enter CH_ERROR would settle it.</t>
+          <t>CHECK BY INSPECTION: Escalation drives the channel into sticky CH_ERROR (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:380), so the green cells are fatal transitions. The map is INDEPENDENT of timeout_enable, and that is worth a look: strikes are cleared only by channel reset, by reaching CH_IDLE, or by real write progress (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:932-936) -- never by the enable bit going low. So a channel that has already accumulated strikes and then has cfg_sched_timeout_enable cleared by software still has w_timeout_escalate asserted and still wedges into CH_ERROR. NOT YET ESTABLISHED whether any host sequence actually clears enable mid-transfer; the map states the exposure rather than asserting the bug. A directed test that raises strikes, clears enable, and checks the channel does not enter CH_ERROR would settle it.</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:965</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:965</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:966</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:966</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:971</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:971</t>
         </is>
       </c>
     </row>
@@ -3734,14 +3734,14 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:970, projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:971</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:970, projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:971</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>DEPENDS ONLY ON: these four. cfg_sched_timeout_cycles enters only through counter_expired; the counter's own 4-way arming priority (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:920-928) decides WHEN a window elapses, not whether escalation fires once strikes are banked.</t>
+          <t>DEPENDS ONLY ON: these four. cfg_sched_timeout_cycles enters only through counter_expired; the counter's own 4-way arming priority (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:920-928) decides WHEN a window elapses, not whether escalation fires once strikes are banked.</t>
         </is>
       </c>
     </row>
@@ -3887,14 +3887,14 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:418</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:418</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>The alloc/drain FUBs are byte-identical between the two projects; this scheduler is not. The divergence is narrow -- one term in the completion wire and the placement of the commit-wait -- but it changes chain behaviour and which descriptor exposes a lost commit. Neither side has a recovery path; see projects/components/dmas/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md, whose section 6a found the write engine byte-identical and therefore the under-count risk shared.</t>
+          <t>The alloc/drain FUBs are byte-identical between the two projects; this scheduler is not. The divergence is narrow -- one term in the completion wire and the placement of the commit-wait -- but it changes chain behaviour and which descriptor exposes a lost commit. Neither side has a recovery path; see projects/components/dma-ip/rapids/known_issues/resolved/snk_scheduler_write_commit_stall.md, whose section 6a found the write engine byte-identical and therefore the under-count risk shared.</t>
         </is>
       </c>
     </row>
@@ -3923,12 +3923,12 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>w_write_issued -- issue-based (projects/components/dmas/stream/rtl/fub/scheduler.sv:909)</t>
+          <t>w_write_issued -- issue-based (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:909)</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>w_write_complete -- commit-based (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:776)</t>
+          <t>w_write_complete -- commit-based (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:776)</t>
         </is>
       </c>
     </row>
@@ -3940,12 +3940,12 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>(w_read_complete &amp;&amp; w_write_issued) (projects/components/dmas/stream/rtl/fub/scheduler.sv:1376)</t>
+          <t>(w_read_complete &amp;&amp; w_write_issued) (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:1376)</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>(w_read_complete &amp;&amp; w_write_complete) (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:1136)</t>
+          <t>(w_read_complete &amp;&amp; w_write_complete) (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:1136)</t>
         </is>
       </c>
     </row>
@@ -3957,12 +3957,12 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>yes, last descriptor only (projects/components/dmas/stream/rtl/fub/scheduler.sv:542); chained advances immediately</t>
+          <t>yes, last descriptor only (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:542); chained advances immediately</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>none (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:424-432)</t>
+          <t>none (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:424-432)</t>
         </is>
       </c>
     </row>
@@ -4008,12 +4008,12 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>same 5 terms (projects/components/dmas/stream/rtl/fub/scheduler.sv:1004-1008)</t>
+          <t>same 5 terms (projects/components/dma-ip/stream/rtl/fub/scheduler.sv:1004-1008)</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>same 5 terms (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:858-862)</t>
+          <t>same 5 terms (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:858-862)</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>rapids TASK-002 items 1 and 2. Item 1: the write engine detects bad B responses per channel, and the sink used to throw that detection away, leaving two fatal-error terms provably dead. FIXED 2026-09-25 -- the maps below show the repaired cone, with the defect kept as a recorded relation so the history is not lost. Item 2: the sink SRAM drain port serves one channel per cycle by construction. Both were filed against retired pre-beats files, so only their anchors were stale; see projects/components/dmas/rapids/known_issues/active/sink_data_path.md and projects/components/dmas/rapids/known_issues/active/sink_sram_control.md.</t>
+          <t>rapids TASK-002 items 1 and 2. Item 1: the write engine detects bad B responses per channel, and the sink used to throw that detection away, leaving two fatal-error terms provably dead. FIXED 2026-09-25 -- the maps below show the repaired cone, with the defect kept as a recorded relation so the history is not lost. Item 2: the sink SRAM drain port serves one channel per cycle by construction. Both were filed against retired pre-beats files, so only their anchors were stale; see projects/components/dma-ip/rapids/known_issues/active/sink_data_path.md and projects/components/dma-ip/rapids/known_issues/active/sink_sram_control.md.</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951 sets it, :955 latches per channel, :964 drives the port declared at :144. The detection is REAL and complete.</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951 sets it, :955 latches per channel, :964 drives the port declared at :144. The detection is REAL and complete.</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:640 connects it, :514 feeds the scheduler_group_array_beats instantiated at :344. The data path exports it at projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_beats.sv:275.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:640 connects it, :514 feeds the scheduler_group_array_beats instantiated at :344. The data path exports it at projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_beats.sv:275.</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:513. Contrast projects/components/dmas/rapids/rtl/macro_beats/rapids_src_beats.sv:491, where the SOURCE wires a real sched_rd_error, and :492 where the source ties its unused write error off for the mirror-image legitimate reason.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:513. Contrast projects/components/dma-ip/rapids/rtl/macro_beats/rapids_src_beats.sv:491, where the SOURCE wires a real sched_rd_error, and :492 where the source ties its unused write error off for the mirror-image legitimate reason.</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:944 latches it, :979 uses it in w_hard_error, :1084 packs it into a monitor packet.</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:944 latches it, :979 uses it in w_hard_error, :1084 packs it into a monitor packet.</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:978-980, consumed at :380. Live terms come from projects/components/dmas/rapids/rtl/macro_beats/scheduler_group_beats.sv:264 (descriptor_engine_beats) and projects/components/dmas/rapids/rtl/fub/ctrlrd_engine.sv:437.</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:978-980, consumed at :380. Live terms come from projects/components/dma-ip/rapids/rtl/macro_beats/scheduler_group_beats.sv:264 (descriptor_engine_beats) and projects/components/dma-ip/rapids/rtl/fub/ctrlrd_engine.sv:437.</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147-148 decode, :157 mux. See projects/components/dmas/rapids/known_issues/active/sink_sram_control.md -- the limitation is structural, which is why a keyword search for "single read" finds nothing.</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147-148 decode, :157 mux. See projects/components/dma-ip/rapids/known_issues/active/sink_sram_control.md -- the limitation is structural, which is why a keyword search for "single read" finds nothing.</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>rapids_snk_beats / scheduler_beats - fatal-error entry (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:978)</t>
+          <t>rapids_snk_beats / scheduler_beats - fatal-error entry (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:978)</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:978</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:978</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: 16 of 32 cells are unreachable, and NOT for the usual reason: they are states the INSTANTIATION forbids by tying an input to a constant, not states that cannot physically occur. The one surviving exclusion is legitimate -- the sink has no AXI read engine, so rd_path is identically 0. Of the 16 reachable cells 15 are green: any single error term faults the channel. COMPARE THE PREVIOUS VERSION: until 2026-09-25 wr_error and wr_sticky were ALSO tied to 0, only 4 cells were reachable, and a SLVERR or DECERR on every beat of a transfer produced no fatal error, no CH_ERROR (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:380) and no error bit in the MonBus packet (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:1084) -- the channel reported success. The detection was always real (projects/components/dmas/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951/:955/:964); only the wiring was missing, and it is now in place.</t>
+          <t>CHECK BY INSPECTION: 16 of 32 cells are unreachable, and NOT for the usual reason: they are states the INSTANTIATION forbids by tying an input to a constant, not states that cannot physically occur. The one surviving exclusion is legitimate -- the sink has no AXI read engine, so rd_path is identically 0. Of the 16 reachable cells 15 are green: any single error term faults the channel. COMPARE THE PREVIOUS VERSION: until 2026-09-25 wr_error and wr_sticky were ALSO tied to 0, only 4 cells were reachable, and a SLVERR or DECERR on every beat of a transfer produced no fatal error, no CH_ERROR (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:380) and no error bit in the MonBus packet (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:1084) -- the channel reported success. The detection was always real (projects/components/dma-ip/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951/:955/:964); only the wiring was missing, and it is now in place.</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/scheduler_group_beats.sv:264, wired :289</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/scheduler_group_beats.sv:264, wired :289</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:163</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:163</t>
         </is>
       </c>
     </row>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:944</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:944</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:162, :943</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:162, :943</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:980, driven projects/components/dmas/rapids/rtl/fub/ctrlrd_engine.sv:437</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:980, driven projects/components/dma-ip/rapids/rtl/fub/ctrlrd_engine.sv:437</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:513</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:513</t>
         </is>
       </c>
     </row>
@@ -4563,14 +4563,14 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:640, path :514 -&gt; projects/components/dmas/rapids/rtl/macro_beats/scheduler_group_array_beats.sv:541 -&gt; projects/components/dmas/rapids/rtl/macro_beats/scheduler_group_beats.sv:411 -&gt; projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:163; exported at projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_beats.sv:275</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:640, path :514 -&gt; projects/components/dma-ip/rapids/rtl/macro_beats/scheduler_group_array_beats.sv:541 -&gt; projects/components/dma-ip/rapids/rtl/macro_beats/scheduler_group_beats.sv:411 -&gt; projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:163; exported at projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_beats.sv:275</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>DEPENDS ONLY ON: these five. The timeout path is a SEPARATE disjunct at the FSM (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:380) and is mapped below; channel reset overrides both.</t>
+          <t>DEPENDS ONLY ON: these five. The timeout path is a SEPARATE disjunct at the FSM (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:380) and is mapped below; channel reset overrides both.</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:380</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:380</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: No cell is excluded here any more: all four routes into sticky CH_ERROR are live on the sink since the wr_error wiring was restored on 2026-09-25. 15 of 16 cells are green -- any one fault takes the channel to CH_ERROR. The wr_error column is the part that was dead: previously every cell with it set was unreachable, so a bad write response could not fault the channel at all. One consequence is worth keeping in view even now: a SLVERR arrives WITH a B response, and the commit strobe is gated on bvalid/bready and BID with no bresp test (projects/components/dmas/rapids/rtl/fub_beats/axi_write_engine_beats.sv:898), so it still counts as write progress and resets the timeout counter (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:920). The error path catches it now. A burst that returns no B at all is a different mechanism and is NOT this cone's job: AXI transaction timeouts are detected by the monitor layer by design (rtl/amba/monitor/axi_monitor_timer.sv plus axi_monitor_reporter_timeout.sv, gated by cfg_timeout_enable), not by a counter in the engine. NOT YET ESTABLISHED: no test drives a sink SLVERR today; a directed test returning SLVERR on one burst and checking the channel faults would close the loop.</t>
+          <t>CHECK BY INSPECTION: No cell is excluded here any more: all four routes into sticky CH_ERROR are live on the sink since the wr_error wiring was restored on 2026-09-25. 15 of 16 cells are green -- any one fault takes the channel to CH_ERROR. The wr_error column is the part that was dead: previously every cell with it set was unreachable, so a bad write response could not fault the channel at all. One consequence is worth keeping in view even now: a SLVERR arrives WITH a B response, and the commit strobe is gated on bvalid/bready and BID with no bresp test (projects/components/dma-ip/rapids/rtl/fub_beats/axi_write_engine_beats.sv:898), so it still counts as write progress and resets the timeout counter (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:920). The error path catches it now. A burst that returns no B at all is a different mechanism and is NOT this cone's job: AXI transaction timeouts are detected by the monitor layer by design (rtl/amba/monitor/axi_monitor_timer.sv plus axi_monitor_reporter_timeout.sv, gated by cfg_timeout_enable), not by a counter in the engine. NOT YET ESTABLISHED: no test drives a sink SLVERR today; a directed test returning SLVERR on one burst and checking the channel faults would close the loop.</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/scheduler_group_beats.sv:289</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/scheduler_group_beats.sv:289</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:163</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:163</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:980</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:980</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:970</t>
         </is>
       </c>
     </row>
@@ -4984,14 +4984,14 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:640</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:640</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>DEPENDS ONLY ON: these four, plus channel reset which takes priority over the whole branch (projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:369-370).</t>
+          <t>DEPENDS ONLY ON: these four, plus channel reset which takes priority over the whole branch (projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:369-370).</t>
         </is>
       </c>
     </row>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>CHECK BY INSPECTION: rapids TASK-002 item 2, and the map states the limitation exactly. Two things are visible. (1) The decode is INDEPENDENT of ch_has_data: a drain is decoded to whichever channel drain_id names, whether or not it holds data -- safety is entirely the consumer's responsibility. (2) More importantly, drain_id is a SINGLE index and drain_read a SINGLE bit, so at most one channel's decode can assert in any cycle. Concurrent drains are excluded by the port shape, not by anything in this expression, which is why searching the module for a 'single read' guard finds nothing -- there is no logic to find. Supporting concurrency would mean widening drain_read/drain_id/drain_data to per-channel vectors. The fill side has the identical shape. This is an architectural simplification, not a bug (projects/components/dmas/rapids/known_issues/active/sink_sram_control.md keeps it Low priority).</t>
+          <t>CHECK BY INSPECTION: rapids TASK-002 item 2, and the map states the limitation exactly. Two things are visible. (1) The decode is INDEPENDENT of ch_has_data: a drain is decoded to whichever channel drain_id names, whether or not it holds data -- safety is entirely the consumer's responsibility. (2) More importantly, drain_id is a SINGLE index and drain_read a SINGLE bit, so at most one channel's decode can assert in any cycle. Concurrent drains are excluded by the port shape, not by anything in this expression, which is why searching the module for a 'single read' guard finds nothing -- there is no logic to find. Supporting concurrency would mean widening drain_read/drain_id/drain_data to per-channel vectors. The fill side has the identical shape. This is an architectural simplification, not a bug (projects/components/dma-ip/rapids/known_issues/active/sink_sram_control.md keeps it Low priority).</t>
         </is>
       </c>
     </row>
@@ -5184,7 +5184,7 @@
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:148</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:148</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:157</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:157</t>
         </is>
       </c>
     </row>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_sram_controller_beats.sv:147</t>
         </is>
       </c>
     </row>
@@ -5407,14 +5407,14 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:640</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:640</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>Applied 2026-09-25, mirroring what the RAPIDS source path (projects/components/dmas/rapids/rtl/macro_beats/rapids_src_beats.sv:491) and STREAM already did. Verilator lint is warning-for-warning identical to the pre-change baseline. Gap 1 of the known issue is NOT fixed: there is still no AXI transaction timeout in axi_write_engine_beats, and that file is byte-identical with STREAM's. See projects/components/dmas/rapids/known_issues/active/sink_data_path.md.</t>
+          <t>Applied 2026-09-25, mirroring what the RAPIDS source path (projects/components/dma-ip/rapids/rtl/macro_beats/rapids_src_beats.sv:491) and STREAM already did. Verilator lint is warning-for-warning identical to the pre-change baseline. Gap 1 of the known issue is NOT fixed: there is still no AXI transaction timeout in axi_write_engine_beats, and that file is byte-identical with STREAM's. See projects/components/dma-ip/rapids/known_issues/active/sink_data_path.md.</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951 / :955 / :964</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/axi_write_engine_beats.sv:951 / :955 / :964</t>
         </is>
       </c>
     </row>
@@ -5465,7 +5465,7 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/snk_data_path_beats.sv:275</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/snk_data_path_beats.sv:275</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/macro_beats/rapids_snk_beats.sv:640 -&gt; :514</t>
+          <t>projects/components/dma-ip/rapids/rtl/macro_beats/rapids_snk_beats.sv:640 -&gt; :514</t>
         </is>
       </c>
     </row>
@@ -5516,7 +5516,7 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/rapids/rtl/fub_beats/scheduler_beats.sv:944 / :979 / :1084</t>
+          <t>projects/components/dma-ip/rapids/rtl/fub_beats/scheduler_beats.sv:944 / :979 / :1084</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>projects/components/dmas/stream/rtl/macro/stream_core.sv:669 / :1047 / :2130</t>
+          <t>projects/components/dma-ip/stream/rtl/macro/stream_core.sv:669 / :1047 / :2130</t>
         </is>
       </c>
     </row>

</xml_diff>